<commit_message>
VT #163: Bloomfield municipal sweep (worked example)
Selectboard (3), Town Treasurer, and Justices of the Peace (5) backfilled from Vermont SOS Elections Division directories, plus the November 5, 2024 JP election record. Town Clerk post created with the membership held (conflicting official directories). Workbook Bloomfield row and Status Log updated. Validation: PASSED, 0 errors.
</commit_message>
<xml_diff>
--- a/reference/VT Rolling Audit/VT_Municipalities.xlsx
+++ b/reference/VT Rolling Audit/VT_Municipalities.xlsx
@@ -3044,27 +3044,27 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>None (no official town website)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>None (general law; no Title 24 Appendix chapter)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>None published</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Needs Research</t>
+          <t>Roster backfilled 2026-10-16</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Added 2026-10-16 (issue #163 fix): missing from the Census 2022 seed; verified on the official Vermont.gov Towns &amp; Cities explorer. Charter/code/website backfill as per sheet.</t>
+          <t>Added 2026-10-16 (issue #163 fix): missing from the Census 2022 seed; verified on the official Vermont.gov Towns &amp; Cities explorer. Municipal sweep completed 2026-10-16 (worked example, tracking PR #168): Selectboard, Town Treasurer, and Justices of the Peace backfilled from SOS Elections Division directories; November 5, 2024 JP election record built. Town Clerk holder HELD (SOS guide, SOS contact spreadsheet, and Vermont.gov explorer name three different people). Lesser town officers await the printed town report or a clerk reply. No charter (general law), no official website, no published code.</t>
         </is>
       </c>
     </row>
@@ -16595,7 +16595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16686,6 +16686,33 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Bloomfield municipal sweep -- worked example for the VT municipal tier (tracking PR #168). Roster backfilled from SOS Elections Division directories: Selectboard -- Eric Brault, Josh Riley, Denault Routhier (SOS selectboard directory, June 5, 2026); Town Treasurer -- Sharon Belknap (SOS treasurer contact spreadsheet, June 12, 2026, corroborated by the SOS clerk guide, January 2026); Justices of the Peace x5 -- Ray Bowen, Sharon Belknap, Bryant Wheeler, Suzanne Routhier, Steven Bunnell (SOS '2025-2026 Vermont Justices of the Peace' listing, December 4, 2025), with the November 5, 2024 JP election record built from the same listing (vote totals not published there and not recorded). Town Clerk membership HELD: the SOS guide (January 2026) names Susan Robidas, the SOS clerk contact spreadsheet (June 2026) names Ray Bowen, and the Vermont.gov explorer names Paulette Routhier -- post created, holder awaits a tiebreak. Moderator, Listers, Auditors, Constables, Grand Juror, and Town Agent were NOT minted: no official online source names Bloomfield's holders (no town website; the printed annual town report is not posted). Charter: none -- no Title 24 Appendix chapter (general-law town, full index checked); no official website; no published municipal code. Factory concordance: the VT Jurisdiction Factory carries Selectboard only for Bloomfield and matches name-for-name; every other office is outside its bounded scope.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Municipalities (Bloomfield row), Status Log</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>VT SOS Elections Division directories (selectboard directory; clerk/treasurer contact spreadsheets; JP listing); Title 24 Appendix chapter index (Vermont Statutes Online)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>CivicMirror</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
VT #163: Bloomfield Town Clerk resolved - Ray Bowen minted
The three-way official-source conflict resolved as older vintages: SOS clerk contact spreadsheet (June 12, 2026) names Bowen, corroborated by a September 1, 2026 directory pull; the SOS Guide (Jan 2026) named Susan Robidas, who held the office into early 2026; the vermont.gov explorer carries a ~2022 listing (Paulette Routhier). Minted at Walter's direction on the existing Ray Bowen person record (also a Justice of the Peace). Workbook updated. Validation: PASSED, 0 errors.
</commit_message>
<xml_diff>
--- a/reference/VT Rolling Audit/VT_Municipalities.xlsx
+++ b/reference/VT Rolling Audit/VT_Municipalities.xlsx
@@ -3064,7 +3064,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Added 2026-10-16 (issue #163 fix): missing from the Census 2022 seed; verified on the official Vermont.gov Towns &amp; Cities explorer. Municipal sweep completed 2026-10-16 (worked example, tracking PR #168): Selectboard, Town Treasurer, and Justices of the Peace backfilled from SOS Elections Division directories; November 5, 2024 JP election record built. Town Clerk holder HELD (SOS guide, SOS contact spreadsheet, and Vermont.gov explorer name three different people). Lesser town officers await the printed town report or a clerk reply. No charter (general law), no official website, no published code.</t>
+          <t>Added 2026-10-16 (issue #163 fix): missing from the Census 2022 seed; verified on the official Vermont.gov Towns &amp; Cities explorer. Municipal sweep completed 2026-10-16 (worked example, tracking PR #168): Selectboard, Town Treasurer, and Justices of the Peace backfilled from SOS Elections Division directories; November 5, 2024 JP election record built. Town Clerk resolved to Ray Bowen (SOS clerk contact spreadsheet, June 2026; the SOS guide's Robidas and the explorer's Routhier listings are stale vintages). Lesser town officers await the printed town report or a clerk reply. No charter (general law), no official website, no published code.</t>
         </is>
       </c>
     </row>
@@ -16595,7 +16595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16713,6 +16713,33 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bloomfield Town Clerk resolved (follow-up to the sweep entry above; tracking PR #168). News/directory check at Walter's request, most recent first: Vermont Attorneys Title clerk directory (data obtained September 1, 2026) names Ray Bowen; the SOS clerk contact spreadsheet (June 12, 2026) names Ray Bowen; the North Star Monthly clerk directory (updated ~April 2026) and the SOS guide (January 2026) name Susan Robidas; VPIRG's clerk list (~2022) names Paulette Routhier -- the vintage the Vermont.gov explorer still carries. No news article covers the change. Walter directed minting Bowen on 2026-10-16: clerk membership added (Bowen already held a Justice of the Peace seat on the same person record). Robidas held the office into early 2026; Routhier's listing is a ~2022 artifact.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Municipalities (Bloomfield row), Status Log</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>VT SOS clerk contact spreadsheet (June 12, 2026); Vermont Attorneys Title town clerk directory (September 1, 2026); North Star Monthly Kingdom Guide clerk directory; VPIRG clerk list (~2022)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>CivicMirror</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
VT #163: Bloomfield data set completed - lesser-office posts added
The five remaining 17 V.S.A. section 2646 town offices are created as structure-only posts (Moderator 1 seat, Listers 3, Auditors 3, Grand Juror 1, Town Agent 1), the posts-first pattern of the state/county build. No official source publishes Bloomfield's current holders for these offices, so memberships await the printed annual town report or a clerk records reply. Constable and Collector of Delinquent Taxes posts are not created: the constable seat count is a per-town vote and the collector is the treasurer ex officio unless the town votes otherwise (section 2651d). Bloomfield totals: 9 posts, 10 memberships, 8 people, 1 election record. Workbook updated. Validation: PASSED, 0 errors.
</commit_message>
<xml_diff>
--- a/reference/VT Rolling Audit/VT_Municipalities.xlsx
+++ b/reference/VT Rolling Audit/VT_Municipalities.xlsx
@@ -3064,7 +3064,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Added 2026-10-16 (issue #163 fix): missing from the Census 2022 seed; verified on the official Vermont.gov Towns &amp; Cities explorer. Municipal sweep completed 2026-10-16 (worked example, tracking PR #168): Selectboard, Town Treasurer, and Justices of the Peace backfilled from SOS Elections Division directories; November 5, 2024 JP election record built. Town Clerk resolved to Ray Bowen (SOS clerk contact spreadsheet, June 2026; the SOS guide's Robidas and the explorer's Routhier listings are stale vintages). Lesser town officers await the printed town report or a clerk reply. No charter (general law), no official website, no published code.</t>
+          <t>Added 2026-10-16 (issue #163 fix): missing from the Census 2022 seed; verified on the official Vermont.gov Towns &amp; Cities explorer. Municipal sweep completed 2026-10-16 (worked example, tracking PR #168): Selectboard, Town Treasurer, and Justices of the Peace backfilled from SOS Elections Division directories; November 5, 2024 JP election record built. Town Clerk resolved to Ray Bowen (SOS clerk contact spreadsheet, June 2026; the SOS guide's Robidas and the explorer's Routhier listings are stale vintages). Lesser town offices (Moderator, Listers x3, Auditors x3, Grand Juror, Town Agent) created as structure-only posts from 17 V.S.A. section 2646; holders await the printed town report or a clerk reply. Constable and Collector of Delinquent Taxes posts not created (per-town variations unverifiable). No charter (general law), no official website, no published code.</t>
         </is>
       </c>
     </row>
@@ -16595,7 +16595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16740,6 +16740,33 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bloomfield data set completed as far as available information allows (tracking PR #168; supersedes the sweep entry's 'not minted' note for five of the six lesser offices). The five remaining section 2646 town offices - Moderator (1 seat), Listers (3), Auditors (3), Grand Juror (1), Town Agent (1) - were created as structure-only posts from 17 V.S.A. section 2646, the posts-first pattern used for the state and county build. No official source publishes Bloomfield's current holders for these offices, so memberships await the printed annual town report or a clerk records reply. Constable and Collector of Delinquent Taxes posts were NOT created: a post requires a seat count, towns elect one or two constables by local vote, and the collector is the treasurer ex officio unless the town votes to elect one separately (section 2651d) - both unverifiable from published sources. A final sweep of the VT Jurisdiction Factory confirmed it carries Bloomfield selectboard data only. Bloomfield totals in the repo: 9 posts, 10 memberships, 8 people, 1 election record.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Municipalities (Bloomfield row), Status Log</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>17 V.S.A. sections 2646, 2649, 2651, 2651b, 2651d (Vermont Statutes Online); VT Jurisdiction Factory v0.1 (coverage re-check 2026-10-16)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>CivicMirror</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>